<commit_message>
Sync Financial Template from main (Lookup Tables header rename)
Pulls 1db7a6c from origin/main, which renames Lookup Tables columns
from "Subtype / Account Type Lookup" to "Account Type / Account Type
Group". Establishes the schema the parser will read for the
Brokerage / Retirement / HSA / ESA sidebar split.

https://claude.ai/code/session_01UAhuywSAPagqMwpdjZvzPo
</commit_message>
<xml_diff>
--- a/core/sample-data/Financial Template.xlsx
+++ b/core/sample-data/Financial Template.xlsx
@@ -3,12 +3,12 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10419"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C139EB28-2D46-0E42-AC68-08019D845E55}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AA9D0CDC-6962-CA41-9F77-944906F846C5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="5040" yWindow="600" windowWidth="23760" windowHeight="14620" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Lookup Tables" sheetId="8" r:id="rId1"/>
+    <sheet name="Lookup Tables" sheetId="8" state="hidden" r:id="rId1"/>
     <sheet name="Accounts" sheetId="4" r:id="rId2"/>
     <sheet name="Net Worth MoM" sheetId="2" r:id="rId3"/>
     <sheet name="Mortgage" sheetId="1" r:id="rId4"/>
@@ -64,7 +64,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="566" uniqueCount="317">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="566" uniqueCount="316">
   <si>
     <t>I captured data at month end balances</t>
   </si>
@@ -969,12 +969,6 @@
     <t>Etta</t>
   </si>
   <si>
-    <t>Subtype</t>
-  </si>
-  <si>
-    <t>Account Type Lookup</t>
-  </si>
-  <si>
     <t>Trust</t>
   </si>
   <si>
@@ -1015,6 +1009,9 @@
   </si>
   <si>
     <t>RSU</t>
+  </si>
+  <si>
+    <t>Account Type Group</t>
   </si>
 </sst>
 </file>
@@ -1483,8 +1480,8 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{23417DED-0198-6143-B962-A0F5AD48A263}" name="Table3" displayName="Table3" ref="B2:C18" totalsRowShown="0" dataDxfId="8">
   <autoFilter ref="B2:C18" xr:uid="{EE18B4AB-3C31-074B-A1AF-5770971F7EB4}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{6C8268AC-5A43-7348-9E49-D23B2435E709}" name="Subtype" dataDxfId="7"/>
-    <tableColumn id="2" xr3:uid="{D8D4C27C-BFF3-F042-8978-1BA496608353}" name="Account Type Lookup" dataDxfId="6"/>
+    <tableColumn id="1" xr3:uid="{6C8268AC-5A43-7348-9E49-D23B2435E709}" name="Account Type" dataDxfId="7"/>
+    <tableColumn id="2" xr3:uid="{D8D4C27C-BFF3-F042-8978-1BA496608353}" name="Account Type Group" dataDxfId="6"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight13" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1812,10 +1809,10 @@
   <sheetData>
     <row r="2" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B2" t="s">
-        <v>301</v>
+        <v>20</v>
       </c>
       <c r="C2" t="s">
-        <v>302</v>
+        <v>315</v>
       </c>
     </row>
     <row r="3" spans="2:3" ht="17" x14ac:dyDescent="0.2">
@@ -1828,7 +1825,7 @@
     </row>
     <row r="4" spans="2:3" ht="17" x14ac:dyDescent="0.2">
       <c r="B4" s="38" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
       <c r="C4" s="38" t="s">
         <v>3</v>
@@ -1836,7 +1833,7 @@
     </row>
     <row r="5" spans="2:3" ht="17" x14ac:dyDescent="0.2">
       <c r="B5" s="38" t="s">
-        <v>304</v>
+        <v>302</v>
       </c>
       <c r="C5" s="38" t="s">
         <v>3</v>
@@ -1844,7 +1841,7 @@
     </row>
     <row r="6" spans="2:3" ht="17" x14ac:dyDescent="0.2">
       <c r="B6" s="38" t="s">
-        <v>305</v>
+        <v>303</v>
       </c>
       <c r="C6" s="38" t="s">
         <v>5</v>
@@ -1852,7 +1849,7 @@
     </row>
     <row r="7" spans="2:3" ht="17" x14ac:dyDescent="0.2">
       <c r="B7" s="38" t="s">
-        <v>306</v>
+        <v>304</v>
       </c>
       <c r="C7" s="38" t="s">
         <v>5</v>
@@ -1860,7 +1857,7 @@
     </row>
     <row r="8" spans="2:3" ht="17" x14ac:dyDescent="0.2">
       <c r="B8" s="38" t="s">
-        <v>307</v>
+        <v>305</v>
       </c>
       <c r="C8" s="38" t="s">
         <v>5</v>
@@ -1868,7 +1865,7 @@
     </row>
     <row r="9" spans="2:3" ht="17" x14ac:dyDescent="0.2">
       <c r="B9" s="38" t="s">
-        <v>308</v>
+        <v>306</v>
       </c>
       <c r="C9" s="38" t="s">
         <v>5</v>
@@ -1876,7 +1873,7 @@
     </row>
     <row r="10" spans="2:3" ht="17" x14ac:dyDescent="0.2">
       <c r="B10" s="38" t="s">
-        <v>309</v>
+        <v>307</v>
       </c>
       <c r="C10" s="38" t="s">
         <v>5</v>
@@ -1884,7 +1881,7 @@
     </row>
     <row r="11" spans="2:3" ht="17" x14ac:dyDescent="0.2">
       <c r="B11" s="38" t="s">
-        <v>310</v>
+        <v>308</v>
       </c>
       <c r="C11" s="38" t="s">
         <v>5</v>
@@ -1892,7 +1889,7 @@
     </row>
     <row r="12" spans="2:3" ht="17" x14ac:dyDescent="0.2">
       <c r="B12" s="38" t="s">
-        <v>311</v>
+        <v>309</v>
       </c>
       <c r="C12" s="38" t="s">
         <v>5</v>
@@ -1900,7 +1897,7 @@
     </row>
     <row r="13" spans="2:3" ht="17" x14ac:dyDescent="0.2">
       <c r="B13" s="38" t="s">
-        <v>312</v>
+        <v>310</v>
       </c>
       <c r="C13" s="38" t="s">
         <v>5</v>
@@ -1908,7 +1905,7 @@
     </row>
     <row r="14" spans="2:3" ht="17" x14ac:dyDescent="0.2">
       <c r="B14" s="38" t="s">
-        <v>313</v>
+        <v>311</v>
       </c>
       <c r="C14" s="38" t="s">
         <v>5</v>
@@ -1927,20 +1924,20 @@
         <v>529</v>
       </c>
       <c r="C16" s="38" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
     </row>
     <row r="17" spans="2:3" ht="17" x14ac:dyDescent="0.2">
       <c r="B17" s="38" t="s">
-        <v>315</v>
+        <v>313</v>
       </c>
       <c r="C17" s="38" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
     </row>
     <row r="18" spans="2:3" ht="17" x14ac:dyDescent="0.2">
       <c r="B18" s="38" t="s">
-        <v>316</v>
+        <v>314</v>
       </c>
       <c r="C18" s="38" t="s">
         <v>3</v>
@@ -1994,7 +1991,7 @@
         <v>38</v>
       </c>
       <c r="C4" s="43" t="s">
-        <v>306</v>
+        <v>304</v>
       </c>
       <c r="D4" s="41" t="s">
         <v>45</v>

</xml_diff>

<commit_message>
Added in Sankey Diagram tool
</commit_message>
<xml_diff>
--- a/core/sample-data/Financial Template.xlsx
+++ b/core/sample-data/Financial Template.xlsx
@@ -3,18 +3,19 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10419"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AA9D0CDC-6962-CA41-9F77-944906F846C5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF0F40E3-EB00-1741-8493-F736B051B236}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5040" yWindow="600" windowWidth="23760" windowHeight="14620" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4300" yWindow="1540" windowWidth="23760" windowHeight="14620" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Lookup Tables" sheetId="8" state="hidden" r:id="rId1"/>
     <sheet name="Accounts" sheetId="4" r:id="rId2"/>
     <sheet name="Net Worth MoM" sheetId="2" r:id="rId3"/>
-    <sheet name="Mortgage" sheetId="1" r:id="rId4"/>
-    <sheet name="Education Savings" sheetId="7" r:id="rId5"/>
-    <sheet name="Brokerage Ledger" sheetId="3" r:id="rId6"/>
-    <sheet name="TICKERS" sheetId="5" r:id="rId7"/>
+    <sheet name="Budget" sheetId="9" r:id="rId4"/>
+    <sheet name="Mortgage" sheetId="1" r:id="rId5"/>
+    <sheet name="Education Savings" sheetId="7" r:id="rId6"/>
+    <sheet name="Brokerage Ledger" sheetId="3" r:id="rId7"/>
+    <sheet name="TICKERS" sheetId="5" r:id="rId8"/>
   </sheets>
   <definedNames>
     <definedName name="APR">#REF!</definedName>
@@ -64,7 +65,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="566" uniqueCount="316">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="617" uniqueCount="342">
   <si>
     <t>I captured data at month end balances</t>
   </si>
@@ -1012,18 +1013,97 @@
   </si>
   <si>
     <t>Account Type Group</t>
+  </si>
+  <si>
+    <t>Source</t>
+  </si>
+  <si>
+    <t>Target</t>
+  </si>
+  <si>
+    <t>Value</t>
+  </si>
+  <si>
+    <t>Emergency '25</t>
+  </si>
+  <si>
+    <t>Emergency OB</t>
+  </si>
+  <si>
+    <t>Dividend Stocks</t>
+  </si>
+  <si>
+    <t>Growth Stocks '25</t>
+  </si>
+  <si>
+    <t>'25 RSUs</t>
+  </si>
+  <si>
+    <t>Investment Reserve</t>
+  </si>
+  <si>
+    <t>WWW OB</t>
+  </si>
+  <si>
+    <t>'25 Cash Bonus</t>
+  </si>
+  <si>
+    <t>Annual OB</t>
+  </si>
+  <si>
+    <t>Travel OB</t>
+  </si>
+  <si>
+    <t>Whatever We Want '25</t>
+  </si>
+  <si>
+    <t>Property Taxes</t>
+  </si>
+  <si>
+    <t>Income Taxes</t>
+  </si>
+  <si>
+    <t>Auto Registrations</t>
+  </si>
+  <si>
+    <t>HOA + Assessment</t>
+  </si>
+  <si>
+    <t>Lila Graduation</t>
+  </si>
+  <si>
+    <t>Ski Trip</t>
+  </si>
+  <si>
+    <t>Kaui</t>
+  </si>
+  <si>
+    <t>Summer Trip(s)</t>
+  </si>
+  <si>
+    <t>Volleyball '26</t>
+  </si>
+  <si>
+    <t>Spring Break '27 Deposit</t>
+  </si>
+  <si>
+    <t>10 Year Mortgage Plan</t>
+  </si>
+  <si>
+    <t>Unallocated</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="5">
+  <numFmts count="6">
     <numFmt numFmtId="8" formatCode="&quot;$&quot;#,##0.00_);[Red]\(&quot;$&quot;#,##0.00\)"/>
     <numFmt numFmtId="164" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="165" formatCode="m/d/yy;@"/>
     <numFmt numFmtId="166" formatCode="\$#,##0.00"/>
     <numFmt numFmtId="167" formatCode="\(\$#,##0.00\);\(\$#,##0.00\)"/>
+    <numFmt numFmtId="168" formatCode="&quot;$&quot;#,##0"/>
   </numFmts>
   <fonts count="14" x14ac:knownFonts="1">
     <font>
@@ -1222,7 +1302,7 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="45">
+  <cellXfs count="46">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1292,6 +1372,7 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="168" fontId="1" fillId="0" borderId="0" xfId="2" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3377,6 +3458,301 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{13E04C96-37C6-B843-8490-73D3F2BBF169}">
+  <sheetPr>
+    <tabColor rgb="FF00B0F0"/>
+  </sheetPr>
+  <dimension ref="B2:D26"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="10.83203125" style="41"/>
+    <col min="2" max="2" width="24" style="41" customWidth="1"/>
+    <col min="3" max="3" width="26" style="41" customWidth="1"/>
+    <col min="4" max="4" width="14" style="41" customWidth="1"/>
+    <col min="5" max="16384" width="10.83203125" style="41"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="2:4" x14ac:dyDescent="0.2">
+      <c r="B2" s="41" t="s">
+        <v>316</v>
+      </c>
+      <c r="C2" s="41" t="s">
+        <v>317</v>
+      </c>
+      <c r="D2" s="41" t="s">
+        <v>318</v>
+      </c>
+    </row>
+    <row r="3" spans="2:4" x14ac:dyDescent="0.2">
+      <c r="B3" s="41" t="s">
+        <v>319</v>
+      </c>
+      <c r="C3" s="41" t="s">
+        <v>320</v>
+      </c>
+      <c r="D3" s="45">
+        <v>45000</v>
+      </c>
+    </row>
+    <row r="4" spans="2:4" x14ac:dyDescent="0.2">
+      <c r="B4" s="41" t="s">
+        <v>46</v>
+      </c>
+      <c r="C4" s="41" t="s">
+        <v>3</v>
+      </c>
+      <c r="D4" s="45">
+        <v>43500</v>
+      </c>
+    </row>
+    <row r="5" spans="2:4" x14ac:dyDescent="0.2">
+      <c r="B5" s="41" t="s">
+        <v>321</v>
+      </c>
+      <c r="C5" s="41" t="s">
+        <v>3</v>
+      </c>
+      <c r="D5" s="45">
+        <v>26500</v>
+      </c>
+    </row>
+    <row r="6" spans="2:4" x14ac:dyDescent="0.2">
+      <c r="B6" s="41" t="s">
+        <v>322</v>
+      </c>
+      <c r="C6" s="41" t="s">
+        <v>3</v>
+      </c>
+      <c r="D6" s="45">
+        <v>537000</v>
+      </c>
+    </row>
+    <row r="7" spans="2:4" x14ac:dyDescent="0.2">
+      <c r="B7" s="41" t="s">
+        <v>323</v>
+      </c>
+      <c r="C7" s="41" t="s">
+        <v>3</v>
+      </c>
+      <c r="D7" s="45">
+        <v>9700</v>
+      </c>
+    </row>
+    <row r="8" spans="2:4" x14ac:dyDescent="0.2">
+      <c r="B8" s="41" t="s">
+        <v>323</v>
+      </c>
+      <c r="C8" s="41" t="s">
+        <v>324</v>
+      </c>
+      <c r="D8" s="45">
+        <v>48500</v>
+      </c>
+    </row>
+    <row r="9" spans="2:4" x14ac:dyDescent="0.2">
+      <c r="B9" s="41" t="s">
+        <v>323</v>
+      </c>
+      <c r="C9" s="41" t="s">
+        <v>325</v>
+      </c>
+      <c r="D9" s="45">
+        <v>18900</v>
+      </c>
+    </row>
+    <row r="10" spans="2:4" x14ac:dyDescent="0.2">
+      <c r="B10" s="41" t="s">
+        <v>324</v>
+      </c>
+      <c r="C10" s="41" t="s">
+        <v>3</v>
+      </c>
+      <c r="D10" s="45">
+        <v>48500</v>
+      </c>
+    </row>
+    <row r="11" spans="2:4" x14ac:dyDescent="0.2">
+      <c r="B11" s="41" t="s">
+        <v>326</v>
+      </c>
+      <c r="C11" s="41" t="s">
+        <v>327</v>
+      </c>
+      <c r="D11" s="45">
+        <v>30700</v>
+      </c>
+    </row>
+    <row r="12" spans="2:4" x14ac:dyDescent="0.2">
+      <c r="B12" s="41" t="s">
+        <v>326</v>
+      </c>
+      <c r="C12" s="41" t="s">
+        <v>328</v>
+      </c>
+      <c r="D12" s="45">
+        <v>49000</v>
+      </c>
+    </row>
+    <row r="13" spans="2:4" x14ac:dyDescent="0.2">
+      <c r="B13" s="41" t="s">
+        <v>326</v>
+      </c>
+      <c r="C13" s="41" t="s">
+        <v>325</v>
+      </c>
+      <c r="D13" s="45">
+        <v>38200</v>
+      </c>
+    </row>
+    <row r="14" spans="2:4" x14ac:dyDescent="0.2">
+      <c r="B14" s="41" t="s">
+        <v>329</v>
+      </c>
+      <c r="C14" s="41" t="s">
+        <v>325</v>
+      </c>
+      <c r="D14" s="45">
+        <v>61200</v>
+      </c>
+    </row>
+    <row r="15" spans="2:4" x14ac:dyDescent="0.2">
+      <c r="B15" s="41" t="s">
+        <v>327</v>
+      </c>
+      <c r="C15" s="41" t="s">
+        <v>330</v>
+      </c>
+      <c r="D15" s="45">
+        <v>14700</v>
+      </c>
+    </row>
+    <row r="16" spans="2:4" x14ac:dyDescent="0.2">
+      <c r="B16" s="41" t="s">
+        <v>327</v>
+      </c>
+      <c r="C16" s="41" t="s">
+        <v>331</v>
+      </c>
+      <c r="D16" s="45">
+        <v>8500</v>
+      </c>
+    </row>
+    <row r="17" spans="2:4" x14ac:dyDescent="0.2">
+      <c r="B17" s="41" t="s">
+        <v>327</v>
+      </c>
+      <c r="C17" s="41" t="s">
+        <v>332</v>
+      </c>
+      <c r="D17" s="45">
+        <v>1500</v>
+      </c>
+    </row>
+    <row r="18" spans="2:4" x14ac:dyDescent="0.2">
+      <c r="B18" s="41" t="s">
+        <v>327</v>
+      </c>
+      <c r="C18" s="41" t="s">
+        <v>333</v>
+      </c>
+      <c r="D18" s="45">
+        <v>2000</v>
+      </c>
+    </row>
+    <row r="19" spans="2:4" x14ac:dyDescent="0.2">
+      <c r="B19" s="41" t="s">
+        <v>327</v>
+      </c>
+      <c r="C19" s="41" t="s">
+        <v>334</v>
+      </c>
+      <c r="D19" s="45">
+        <v>4000</v>
+      </c>
+    </row>
+    <row r="20" spans="2:4" x14ac:dyDescent="0.2">
+      <c r="B20" s="41" t="s">
+        <v>328</v>
+      </c>
+      <c r="C20" s="41" t="s">
+        <v>335</v>
+      </c>
+      <c r="D20" s="45">
+        <v>4000</v>
+      </c>
+    </row>
+    <row r="21" spans="2:4" x14ac:dyDescent="0.2">
+      <c r="B21" s="41" t="s">
+        <v>328</v>
+      </c>
+      <c r="C21" s="41" t="s">
+        <v>336</v>
+      </c>
+      <c r="D21" s="45">
+        <v>5000</v>
+      </c>
+    </row>
+    <row r="22" spans="2:4" x14ac:dyDescent="0.2">
+      <c r="B22" s="41" t="s">
+        <v>328</v>
+      </c>
+      <c r="C22" s="41" t="s">
+        <v>337</v>
+      </c>
+      <c r="D22" s="45">
+        <v>21000</v>
+      </c>
+    </row>
+    <row r="23" spans="2:4" x14ac:dyDescent="0.2">
+      <c r="B23" s="41" t="s">
+        <v>328</v>
+      </c>
+      <c r="C23" s="41" t="s">
+        <v>338</v>
+      </c>
+      <c r="D23" s="45">
+        <v>4000</v>
+      </c>
+    </row>
+    <row r="24" spans="2:4" x14ac:dyDescent="0.2">
+      <c r="B24" s="41" t="s">
+        <v>328</v>
+      </c>
+      <c r="C24" s="41" t="s">
+        <v>339</v>
+      </c>
+      <c r="D24" s="45">
+        <v>15000</v>
+      </c>
+    </row>
+    <row r="25" spans="2:4" x14ac:dyDescent="0.2">
+      <c r="B25" s="41" t="s">
+        <v>325</v>
+      </c>
+      <c r="C25" s="41" t="s">
+        <v>340</v>
+      </c>
+      <c r="D25" s="45">
+        <v>38400</v>
+      </c>
+    </row>
+    <row r="26" spans="2:4" x14ac:dyDescent="0.2">
+      <c r="B26" s="41" t="s">
+        <v>325</v>
+      </c>
+      <c r="C26" s="41" t="s">
+        <v>341</v>
+      </c>
+      <c r="D26" s="45">
+        <v>80100</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <sheetPr>
     <tabColor rgb="FF00B0F0"/>
@@ -3443,7 +3819,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BBB0E85D-0232-5647-9A75-FF64DBBA5AC5}">
   <sheetPr>
     <tabColor theme="8"/>
@@ -5342,7 +5718,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr>
     <tabColor theme="8"/>
@@ -8771,7 +9147,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <sheetPr>
     <tabColor theme="8"/>

</xml_diff>